<commit_message>
feature added: read data from DB and save result to DB
</commit_message>
<xml_diff>
--- a/Test_DemoWebShop/Result/OrderDetails.xlsx
+++ b/Test_DemoWebShop/Result/OrderDetails.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riseup\Katalon Studio\Test_Demo\Result\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Riseup\Katalon Studio\Test_DemoWebShop\Result\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF03634-F6E5-4BC0-AA34-23106BE9D86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FC8C49-9B96-48CD-B7FB-501002EBB44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Order Number</t>
   </si>
@@ -43,12 +43,55 @@
   </si>
   <si>
     <t>PDF Download Status</t>
+  </si>
+  <si>
+    <t>2323543</t>
+  </si>
+  <si>
+    <t>Login Successful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">These items were added to cart- Fiction:2, Health Book:3, Computing and Internet:1, </t>
+  </si>
+  <si>
+    <t>Next Day Air</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>downloaded order_2323543.pdf</t>
+  </si>
+  <si>
+    <t>2323545</t>
+  </si>
+  <si>
+    <t xml:space="preserve">These items were added to cart- Blue Jeans:2, Blue and green Sneaker:3, Casual Golf Belt:4, </t>
+  </si>
+  <si>
+    <t>2nd Day Air</t>
+  </si>
+  <si>
+    <t>downloaded order_2323545.pdf</t>
+  </si>
+  <si>
+    <t>2323754</t>
+  </si>
+  <si>
+    <t>downloaded order_2323754.pdf</t>
+  </si>
+  <si>
+    <t>2323755</t>
+  </si>
+  <si>
+    <t>downloaded order_2323755.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -360,35 +403,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" customWidth="1"/>
-    <col min="3" max="3" width="75.21875" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" customWidth="1"/>
-    <col min="6" max="6" width="31.88671875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="12.6640625"/>
+    <col min="2" max="2" customWidth="true" width="14.88671875"/>
+    <col min="3" max="3" customWidth="true" width="75.21875"/>
+    <col min="4" max="4" customWidth="true" width="14.44140625"/>
+    <col min="5" max="5" customWidth="true" width="11.109375"/>
+    <col min="6" max="6" customWidth="true" width="31.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added pdf data verification function
</commit_message>
<xml_diff>
--- a/Test_DemoWebShop/Result/OrderDetails.xlsx
+++ b/Test_DemoWebShop/Result/OrderDetails.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
   <si>
     <t>Order Number</t>
   </si>
@@ -85,6 +85,42 @@
   </si>
   <si>
     <t>downloaded order_2323755.pdf</t>
+  </si>
+  <si>
+    <t>2325346</t>
+  </si>
+  <si>
+    <t>downloaded order_2325346.pdf</t>
+  </si>
+  <si>
+    <t>2325364</t>
+  </si>
+  <si>
+    <t>downloaded order_2325364.pdf</t>
+  </si>
+  <si>
+    <t>2325391</t>
+  </si>
+  <si>
+    <t>downloaded order_2325391.pdf</t>
+  </si>
+  <si>
+    <t>2325393</t>
+  </si>
+  <si>
+    <t>downloaded order_2325393.pdf</t>
+  </si>
+  <si>
+    <t>2326008</t>
+  </si>
+  <si>
+    <t>downloaded order_2326008.pdf</t>
+  </si>
+  <si>
+    <t>2326009</t>
+  </si>
+  <si>
+    <t>downloaded order_2326009.pdf</t>
   </si>
 </sst>
 </file>
@@ -403,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="12.6640625"/>
@@ -514,6 +550,126 @@
         <v>19</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>